<commit_message>
test(test-data): update excel test cases and test data across modules
</commit_message>
<xml_diff>
--- a/swarajya-create/consultant-management/test_data/Create-Consultant-Management.xlsx
+++ b/swarajya-create/consultant-management/test_data/Create-Consultant-Management.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -741,7 +741,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
@@ -800,7 +800,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -2486,7 +2486,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>To Be Automated</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">

</xml_diff>